<commit_message>
Task 0 complete: DAR chapter bindings, foresight method, candidate rule
Model file now carries dar_outline (11 chapters, each binding the evidence it
may cite), derived_sources, foresight (unratified, three named steps,
milestone binding) and candidate_indicators.

Chapter 5 binds no pillar and states plainly that DAMM holds no cost, budget
or financing data — the chapter most likely to fabricate is the one now least
able to cite.

Parity test 276 -> 293 checks, negative-controlled against five injected
violations. Verification 76/76. Thread 2 handoff updated to start at the
vendor audition.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gauntlet/loop-1/workbooks-v1.7/DAMM-v1.7-Scoring-Workbook-Blank-Template.xlsx
+++ b/gauntlet/loop-1/workbooks-v1.7/DAMM-v1.7-Scoring-Workbook-Blank-Template.xlsx
@@ -1622,11 +1622,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="6665506"/>
-        <c:axId val="11392902"/>
+        <c:axId val="79507874"/>
+        <c:axId val="22852945"/>
       </c:radarChart>
       <c:catAx>
-        <c:axId val="6665506"/>
+        <c:axId val="79507874"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1656,7 +1656,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11392902"/>
+        <c:crossAx val="22852945"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1664,7 +1664,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11392902"/>
+        <c:axId val="22852945"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="5"/>
@@ -1709,7 +1709,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6665506"/>
+        <c:crossAx val="79507874"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1908,11 +1908,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="17625886"/>
-        <c:axId val="45784829"/>
+        <c:axId val="70145618"/>
+        <c:axId val="77959666"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="17625886"/>
+        <c:axId val="70145618"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1945,7 +1945,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45784829"/>
+        <c:crossAx val="77959666"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1953,7 +1953,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="45784829"/>
+        <c:axId val="77959666"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1996,7 +1996,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17625886"/>
+        <c:crossAx val="70145618"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2570,11 +2570,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="55453798"/>
-        <c:axId val="6835817"/>
+        <c:axId val="98554860"/>
+        <c:axId val="54423133"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="55453798"/>
+        <c:axId val="98554860"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2607,7 +2607,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6835817"/>
+        <c:crossAx val="54423133"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2615,7 +2615,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6835817"/>
+        <c:axId val="54423133"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2658,7 +2658,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55453798"/>
+        <c:crossAx val="98554860"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2848,11 +2848,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="63509903"/>
-        <c:axId val="76397339"/>
+        <c:axId val="67698736"/>
+        <c:axId val="94100958"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="63509903"/>
+        <c:axId val="67698736"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2885,7 +2885,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76397339"/>
+        <c:crossAx val="94100958"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2893,7 +2893,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="76397339"/>
+        <c:axId val="94100958"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="5"/>
@@ -2937,7 +2937,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63509903"/>
+        <c:crossAx val="67698736"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3145,11 +3145,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="97570060"/>
-        <c:axId val="74248808"/>
+        <c:axId val="14411340"/>
+        <c:axId val="3289204"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="97570060"/>
+        <c:axId val="14411340"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3182,7 +3182,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74248808"/>
+        <c:crossAx val="3289204"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3190,7 +3190,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="74248808"/>
+        <c:axId val="3289204"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3233,7 +3233,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97570060"/>
+        <c:crossAx val="14411340"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3513,11 +3513,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="2973012"/>
-        <c:axId val="44291716"/>
+        <c:axId val="19598522"/>
+        <c:axId val="16185674"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2973012"/>
+        <c:axId val="19598522"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3550,7 +3550,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44291716"/>
+        <c:crossAx val="16185674"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3558,7 +3558,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="44291716"/>
+        <c:axId val="16185674"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3601,7 +3601,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2973012"/>
+        <c:crossAx val="19598522"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>